<commit_message>
Ajout de la donnée Sise - code diplôme intermédiaire
</commit_message>
<xml_diff>
--- a/maquette-type.xlsx
+++ b/maquette-type.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apereir\Desktop\En cours\En cours Maquettes\scripts\maquettes-xl2json\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apereir\Documents\En cours\En cours Maquettes\scripts\maquettes-xl2json\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4E7359-D87B-47A2-BD63-BB6F05BCB5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E644C205-C610-4A76-A892-2B137B2B4E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{A6F31FBE-6D40-488E-B868-E7547D61F047}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A6F31FBE-6D40-488E-B868-E7547D61F047}"/>
   </bookViews>
   <sheets>
     <sheet name="Format complet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Format complet'!$A$1:$AV$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Format complet'!$A$1:$AW$2</definedName>
     <definedName name="Ordre">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,12 +33,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="202">
   <si>
     <t>EC</t>
   </si>
@@ -647,6 +650,9 @@
   </si>
   <si>
     <t>Relation au nœud parent : VRAI/FAUX (valeur par défaut : VRAI)</t>
+  </si>
+  <si>
+    <t>SISE - code diplôme intermédiaire</t>
   </si>
 </sst>
 </file>
@@ -1233,6 +1239,18 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1251,18 +1269,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1277,9 +1283,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1317,7 +1323,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1423,7 +1429,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1565,7 +1571,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1573,41 +1579,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{344DF7D5-D639-4355-89FB-833EF1843A63}">
-  <dimension ref="A1:AV47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.2" customHeight="1"/>
+  <dimension ref="A1:AW47"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16.149999999999999" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="55.33203125" customWidth="1"/>
-    <col min="5" max="5" width="60.109375" style="13" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.6640625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="24.6640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="55.28515625" customWidth="1"/>
+    <col min="5" max="5" width="60.140625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="14.33203125" customWidth="1"/>
-    <col min="12" max="12" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.5546875" style="4" customWidth="1"/>
-    <col min="18" max="21" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="14.6640625" style="4" customWidth="1"/>
-    <col min="24" max="30" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.33203125" style="4" customWidth="1"/>
-    <col min="32" max="32" width="19.5546875" style="4" customWidth="1"/>
-    <col min="33" max="33" width="17.44140625" style="4" customWidth="1"/>
-    <col min="34" max="34" width="19.5546875" style="4" customWidth="1"/>
-    <col min="35" max="36" width="17" style="4" customWidth="1"/>
-    <col min="37" max="38" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.44140625" style="4" customWidth="1"/>
-    <col min="40" max="40" width="19.5546875" style="4" customWidth="1"/>
-    <col min="41" max="41" width="22.33203125" style="4" customWidth="1"/>
-    <col min="42" max="42" width="19.44140625" style="4" customWidth="1"/>
-    <col min="43" max="48" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="16.33203125" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="16" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.5703125" style="4" customWidth="1"/>
+    <col min="18" max="21" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="14.7109375" style="4" customWidth="1"/>
+    <col min="24" max="26" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.28515625" style="4" customWidth="1"/>
+    <col min="28" max="31" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="19.28515625" style="4" customWidth="1"/>
+    <col min="33" max="33" width="19.5703125" style="4" customWidth="1"/>
+    <col min="34" max="34" width="17.42578125" style="4" customWidth="1"/>
+    <col min="35" max="35" width="19.5703125" style="4" customWidth="1"/>
+    <col min="36" max="37" width="17" style="4" customWidth="1"/>
+    <col min="38" max="39" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20.42578125" style="4" customWidth="1"/>
+    <col min="41" max="41" width="19.5703125" style="4" customWidth="1"/>
+    <col min="42" max="42" width="22.28515625" style="4" customWidth="1"/>
+    <col min="43" max="43" width="19.42578125" style="4" customWidth="1"/>
+    <col min="44" max="49" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="13" customFormat="1" ht="43.2">
+    <row r="1" spans="1:49" s="13" customFormat="1" ht="63" customHeight="1">
       <c r="A1" s="36" t="s">
         <v>188</v>
       </c>
@@ -1687,73 +1695,76 @@
         <v>50</v>
       </c>
       <c r="AA1" s="37" t="s">
+        <v>201</v>
+      </c>
+      <c r="AB1" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="AB1" s="37" t="s">
+      <c r="AC1" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="AC1" s="37" t="s">
+      <c r="AD1" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="AD1" s="38" t="s">
+      <c r="AE1" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="AE1" s="37" t="s">
+      <c r="AF1" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="AF1" s="37" t="s">
+      <c r="AG1" s="37" t="s">
         <v>181</v>
       </c>
-      <c r="AG1" s="37" t="s">
+      <c r="AH1" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="AH1" s="37" t="s">
+      <c r="AI1" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="AI1" s="37" t="s">
+      <c r="AJ1" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="AJ1" s="37" t="s">
+      <c r="AK1" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="AK1" s="37" t="s">
+      <c r="AL1" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="AL1" s="37" t="s">
+      <c r="AM1" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AM1" s="37" t="s">
+      <c r="AN1" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="AN1" s="37" t="s">
+      <c r="AO1" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AO1" s="37" t="s">
+      <c r="AP1" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="AP1" s="37" t="s">
+      <c r="AQ1" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="AQ1" s="37" t="s">
+      <c r="AR1" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="AR1" s="37" t="s">
+      <c r="AS1" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AS1" s="37" t="s">
+      <c r="AT1" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="AT1" s="37" t="s">
+      <c r="AU1" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="AU1" s="37" t="s">
+      <c r="AV1" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="AV1" s="37" t="s">
+      <c r="AW1" s="37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:48" s="13" customFormat="1" ht="57.6">
+    <row r="2" spans="1:49" s="13" customFormat="1" ht="75">
       <c r="A2" s="39" t="s">
         <v>22</v>
       </c>
@@ -1839,31 +1850,31 @@
         <v>52</v>
       </c>
       <c r="AC2" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD2" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="AD2" s="41" t="s">
+      <c r="AE2" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="AE2" s="40" t="s">
+      <c r="AF2" s="40" t="s">
         <v>189</v>
       </c>
-      <c r="AF2" s="40" t="s">
+      <c r="AG2" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="AG2" s="40" t="s">
+      <c r="AH2" s="40" t="s">
         <v>187</v>
       </c>
-      <c r="AH2" s="40" t="s">
+      <c r="AI2" s="40" t="s">
         <v>192</v>
       </c>
-      <c r="AI2" s="40" t="s">
+      <c r="AJ2" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="AJ2" s="40" t="s">
+      <c r="AK2" s="40" t="s">
         <v>183</v>
-      </c>
-      <c r="AK2" s="40" t="s">
-        <v>51</v>
       </c>
       <c r="AL2" s="40" t="s">
         <v>51</v>
@@ -1872,10 +1883,10 @@
         <v>51</v>
       </c>
       <c r="AN2" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO2" s="40" t="s">
         <v>27</v>
-      </c>
-      <c r="AO2" s="40" t="s">
-        <v>51</v>
       </c>
       <c r="AP2" s="40" t="s">
         <v>51</v>
@@ -1884,10 +1895,10 @@
         <v>51</v>
       </c>
       <c r="AR2" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="AS2" s="40" t="s">
         <v>17</v>
-      </c>
-      <c r="AS2" s="40" t="s">
-        <v>51</v>
       </c>
       <c r="AT2" s="40" t="s">
         <v>51</v>
@@ -1898,8 +1909,11 @@
       <c r="AV2" s="40" t="s">
         <v>51</v>
       </c>
+      <c r="AW2" s="40" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="3" spans="1:48" s="13" customFormat="1" ht="16.2" customHeight="1">
+    <row r="3" spans="1:49" s="13" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A3" s="33"/>
       <c r="B3" s="33"/>
       <c r="C3" s="33"/>
@@ -1948,8 +1962,9 @@
       <c r="AT3" s="33"/>
       <c r="AU3" s="33"/>
       <c r="AV3" s="33"/>
+      <c r="AW3" s="33"/>
     </row>
-    <row r="4" spans="1:48" s="13" customFormat="1" ht="57.6" customHeight="1">
+    <row r="4" spans="1:49" s="13" customFormat="1" ht="57.6" customHeight="1">
       <c r="A4" s="29" t="s">
         <v>69</v>
       </c>
@@ -2011,64 +2026,67 @@
         <v>1000218</v>
       </c>
       <c r="AA4" s="28">
+        <v>1000218</v>
+      </c>
+      <c r="AB4" s="28">
         <v>2</v>
       </c>
-      <c r="AB4" s="28" t="s">
+      <c r="AC4" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="AC4" s="28" t="b">
+      <c r="AD4" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="AD4" s="28" t="str">
+      <c r="AE4" s="28" t="str">
         <f>"02"</f>
         <v>02</v>
       </c>
-      <c r="AE4" s="28" t="s">
+      <c r="AF4" s="28" t="s">
         <v>190</v>
       </c>
-      <c r="AF4" s="28"/>
       <c r="AG4" s="28"/>
       <c r="AH4" s="28"/>
       <c r="AI4" s="28"/>
       <c r="AJ4" s="28"/>
-      <c r="AK4" s="29" t="s">
+      <c r="AK4" s="28"/>
+      <c r="AL4" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="AL4" s="29" t="s">
+      <c r="AM4" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="AM4" s="29" t="s">
+      <c r="AN4" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="AN4" s="29" t="b">
+      <c r="AO4" s="29" t="b">
         <v>1</v>
       </c>
-      <c r="AO4" s="29" t="s">
+      <c r="AP4" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="AP4" s="29" t="s">
+      <c r="AQ4" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="AQ4" s="29" t="s">
+      <c r="AR4" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AR4" s="28">
+      <c r="AS4" s="28">
         <v>4</v>
       </c>
-      <c r="AS4" s="29" t="s">
+      <c r="AT4" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="AT4" s="29" t="s">
+      <c r="AU4" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="AU4" s="29" t="s">
+      <c r="AV4" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="AV4" s="29" t="s">
+      <c r="AW4" s="29" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:48" ht="16.2" customHeight="1">
+    <row r="5" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -2077,7 +2095,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
     </row>
-    <row r="6" spans="1:48" ht="22.95" customHeight="1">
+    <row r="6" spans="1:49" ht="22.9" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>72</v>
       </c>
@@ -2142,8 +2160,9 @@
       <c r="AT6" s="7"/>
       <c r="AU6" s="7"/>
       <c r="AV6" s="7"/>
+      <c r="AW6" s="7"/>
     </row>
-    <row r="7" spans="1:48" ht="24" customHeight="1">
+    <row r="7" spans="1:49" ht="24" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>76</v>
       </c>
@@ -2206,8 +2225,9 @@
       <c r="AT7" s="9"/>
       <c r="AU7" s="9"/>
       <c r="AV7" s="9"/>
+      <c r="AW7" s="9"/>
     </row>
-    <row r="8" spans="1:48" ht="16.2" customHeight="1">
+    <row r="8" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>67</v>
       </c>
@@ -2253,8 +2273,8 @@
       <c r="AE8" s="17"/>
       <c r="AF8" s="17"/>
       <c r="AG8" s="17"/>
-      <c r="AH8" s="31"/>
-      <c r="AI8" s="17"/>
+      <c r="AH8" s="17"/>
+      <c r="AI8" s="31"/>
       <c r="AJ8" s="17"/>
       <c r="AK8" s="17"/>
       <c r="AL8" s="17"/>
@@ -2268,8 +2288,9 @@
       <c r="AT8" s="17"/>
       <c r="AU8" s="17"/>
       <c r="AV8" s="17"/>
+      <c r="AW8" s="17"/>
     </row>
-    <row r="9" spans="1:48" ht="16.2" customHeight="1">
+    <row r="9" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A9" s="21" t="s">
         <v>0</v>
       </c>
@@ -2315,9 +2336,9 @@
       <c r="AC9" s="18"/>
       <c r="AD9" s="18"/>
       <c r="AE9" s="18"/>
-      <c r="AG9" s="18"/>
-      <c r="AH9" s="32"/>
-      <c r="AJ9" s="18"/>
+      <c r="AF9" s="18"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="32"/>
       <c r="AK9" s="18"/>
       <c r="AL9" s="18"/>
       <c r="AM9" s="18"/>
@@ -2330,8 +2351,9 @@
       <c r="AT9" s="18"/>
       <c r="AU9" s="18"/>
       <c r="AV9" s="18"/>
+      <c r="AW9" s="18"/>
     </row>
-    <row r="10" spans="1:48" ht="16.2" customHeight="1">
+    <row r="10" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A10" s="21" t="s">
         <v>0</v>
       </c>
@@ -2394,8 +2416,9 @@
       <c r="AT10" s="18"/>
       <c r="AU10" s="18"/>
       <c r="AV10" s="18"/>
+      <c r="AW10" s="18"/>
     </row>
-    <row r="11" spans="1:48" ht="16.2" customHeight="1">
+    <row r="11" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A11" s="21" t="s">
         <v>0</v>
       </c>
@@ -2456,8 +2479,9 @@
       <c r="AT11" s="18"/>
       <c r="AU11" s="18"/>
       <c r="AV11" s="18"/>
+      <c r="AW11" s="18"/>
     </row>
-    <row r="12" spans="1:48" ht="16.2" customHeight="1">
+    <row r="12" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A12" s="21" t="s">
         <v>0</v>
       </c>
@@ -2520,8 +2544,9 @@
       <c r="AT12" s="18"/>
       <c r="AU12" s="18"/>
       <c r="AV12" s="18"/>
+      <c r="AW12" s="18"/>
     </row>
-    <row r="13" spans="1:48" ht="16.2" customHeight="1">
+    <row r="13" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A13" s="21" t="s">
         <v>0</v>
       </c>
@@ -2582,8 +2607,9 @@
       <c r="AT13" s="18"/>
       <c r="AU13" s="18"/>
       <c r="AV13" s="18"/>
+      <c r="AW13" s="18"/>
     </row>
-    <row r="14" spans="1:48" ht="16.2" customHeight="1">
+    <row r="14" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A14" s="21" t="s">
         <v>0</v>
       </c>
@@ -2644,8 +2670,9 @@
       <c r="AT14" s="18"/>
       <c r="AU14" s="18"/>
       <c r="AV14" s="18"/>
+      <c r="AW14" s="18"/>
     </row>
-    <row r="15" spans="1:48" ht="16.2" customHeight="1">
+    <row r="15" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>67</v>
       </c>
@@ -2708,8 +2735,9 @@
       <c r="AT15" s="17"/>
       <c r="AU15" s="17"/>
       <c r="AV15" s="17"/>
+      <c r="AW15" s="17"/>
     </row>
-    <row r="16" spans="1:48" ht="16.2" customHeight="1">
+    <row r="16" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A16" s="21" t="s">
         <v>0</v>
       </c>
@@ -2772,8 +2800,9 @@
       <c r="AT16" s="18"/>
       <c r="AU16" s="18"/>
       <c r="AV16" s="18"/>
+      <c r="AW16" s="18"/>
     </row>
-    <row r="17" spans="1:48" ht="30" customHeight="1">
+    <row r="17" spans="1:49" ht="30" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>67</v>
       </c>
@@ -2838,8 +2867,9 @@
       <c r="AT17" s="17"/>
       <c r="AU17" s="17"/>
       <c r="AV17" s="17"/>
+      <c r="AW17" s="17"/>
     </row>
-    <row r="18" spans="1:48" ht="15.6">
+    <row r="18" spans="1:49" ht="15.75">
       <c r="A18" s="23" t="s">
         <v>103</v>
       </c>
@@ -2902,8 +2932,9 @@
       <c r="AT18" s="18"/>
       <c r="AU18" s="18"/>
       <c r="AV18" s="18"/>
+      <c r="AW18" s="18"/>
     </row>
-    <row r="19" spans="1:48" ht="31.2">
+    <row r="19" spans="1:49" ht="31.5">
       <c r="A19" s="21" t="s">
         <v>0</v>
       </c>
@@ -2966,8 +2997,9 @@
       <c r="AT19" s="18"/>
       <c r="AU19" s="18"/>
       <c r="AV19" s="18"/>
+      <c r="AW19" s="18"/>
     </row>
-    <row r="20" spans="1:48" ht="16.2" customHeight="1">
+    <row r="20" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A20" s="21" t="s">
         <v>0</v>
       </c>
@@ -3028,8 +3060,9 @@
       <c r="AT20" s="18"/>
       <c r="AU20" s="18"/>
       <c r="AV20" s="18"/>
+      <c r="AW20" s="18"/>
     </row>
-    <row r="21" spans="1:48" ht="16.2" customHeight="1">
+    <row r="21" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A21" s="21" t="s">
         <v>0</v>
       </c>
@@ -3090,8 +3123,9 @@
       <c r="AT21" s="18"/>
       <c r="AU21" s="18"/>
       <c r="AV21" s="18"/>
+      <c r="AW21" s="18"/>
     </row>
-    <row r="22" spans="1:48" ht="16.2" customHeight="1">
+    <row r="22" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A22" s="21" t="s">
         <v>0</v>
       </c>
@@ -3152,8 +3186,9 @@
       <c r="AT22" s="18"/>
       <c r="AU22" s="18"/>
       <c r="AV22" s="18"/>
+      <c r="AW22" s="18"/>
     </row>
-    <row r="23" spans="1:48" ht="31.2">
+    <row r="23" spans="1:49" ht="31.5">
       <c r="A23" s="21" t="s">
         <v>0</v>
       </c>
@@ -3216,8 +3251,9 @@
       <c r="AT23" s="18"/>
       <c r="AU23" s="18"/>
       <c r="AV23" s="18"/>
+      <c r="AW23" s="18"/>
     </row>
-    <row r="24" spans="1:48" ht="24" customHeight="1">
+    <row r="24" spans="1:49" ht="24" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>76</v>
       </c>
@@ -3280,8 +3316,9 @@
       <c r="AT24" s="9"/>
       <c r="AU24" s="9"/>
       <c r="AV24" s="9"/>
+      <c r="AW24" s="9"/>
     </row>
-    <row r="25" spans="1:48" ht="16.2" customHeight="1">
+    <row r="25" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>67</v>
       </c>
@@ -3344,8 +3381,9 @@
       <c r="AT25" s="17"/>
       <c r="AU25" s="17"/>
       <c r="AV25" s="17"/>
+      <c r="AW25" s="17"/>
     </row>
-    <row r="26" spans="1:48" ht="16.2" customHeight="1">
+    <row r="26" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A26" s="21" t="s">
         <v>0</v>
       </c>
@@ -3406,8 +3444,9 @@
       <c r="AT26" s="18"/>
       <c r="AU26" s="18"/>
       <c r="AV26" s="18"/>
+      <c r="AW26" s="18"/>
     </row>
-    <row r="27" spans="1:48" ht="16.2" customHeight="1">
+    <row r="27" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A27" s="21" t="s">
         <v>0</v>
       </c>
@@ -3470,8 +3509,9 @@
       <c r="AT27" s="18"/>
       <c r="AU27" s="18"/>
       <c r="AV27" s="18"/>
+      <c r="AW27" s="18"/>
     </row>
-    <row r="28" spans="1:48" ht="16.2" customHeight="1">
+    <row r="28" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A28" s="21" t="s">
         <v>0</v>
       </c>
@@ -3532,8 +3572,9 @@
       <c r="AT28" s="18"/>
       <c r="AU28" s="18"/>
       <c r="AV28" s="18"/>
+      <c r="AW28" s="18"/>
     </row>
-    <row r="29" spans="1:48" ht="16.2" customHeight="1">
+    <row r="29" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A29" s="21" t="s">
         <v>0</v>
       </c>
@@ -3596,8 +3637,9 @@
       <c r="AT29" s="18"/>
       <c r="AU29" s="18"/>
       <c r="AV29" s="18"/>
+      <c r="AW29" s="18"/>
     </row>
-    <row r="30" spans="1:48" ht="16.2" customHeight="1">
+    <row r="30" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A30" s="21" t="s">
         <v>0</v>
       </c>
@@ -3658,8 +3700,9 @@
       <c r="AT30" s="18"/>
       <c r="AU30" s="18"/>
       <c r="AV30" s="18"/>
+      <c r="AW30" s="18"/>
     </row>
-    <row r="31" spans="1:48" ht="16.2" customHeight="1">
+    <row r="31" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A31" s="21" t="s">
         <v>0</v>
       </c>
@@ -3720,8 +3763,9 @@
       <c r="AT31" s="18"/>
       <c r="AU31" s="18"/>
       <c r="AV31" s="18"/>
+      <c r="AW31" s="18"/>
     </row>
-    <row r="32" spans="1:48" ht="16.2" customHeight="1">
+    <row r="32" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A32" s="3" t="s">
         <v>67</v>
       </c>
@@ -3784,8 +3828,9 @@
       <c r="AT32" s="17"/>
       <c r="AU32" s="17"/>
       <c r="AV32" s="17"/>
+      <c r="AW32" s="17"/>
     </row>
-    <row r="33" spans="1:48" ht="16.2" customHeight="1">
+    <row r="33" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A33" s="21" t="s">
         <v>0</v>
       </c>
@@ -3848,8 +3893,9 @@
       <c r="AT33" s="18"/>
       <c r="AU33" s="18"/>
       <c r="AV33" s="18"/>
+      <c r="AW33" s="18"/>
     </row>
-    <row r="34" spans="1:48" ht="16.2" customHeight="1">
+    <row r="34" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A34" s="21" t="s">
         <v>0</v>
       </c>
@@ -3912,8 +3958,9 @@
       <c r="AT34" s="18"/>
       <c r="AU34" s="18"/>
       <c r="AV34" s="18"/>
+      <c r="AW34" s="18"/>
     </row>
-    <row r="35" spans="1:48" ht="31.2">
+    <row r="35" spans="1:49" ht="31.5">
       <c r="A35" s="3" t="s">
         <v>67</v>
       </c>
@@ -3978,8 +4025,9 @@
       <c r="AT35" s="17"/>
       <c r="AU35" s="17"/>
       <c r="AV35" s="17"/>
+      <c r="AW35" s="17"/>
     </row>
-    <row r="36" spans="1:48" ht="16.2" customHeight="1">
+    <row r="36" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A36" s="23" t="s">
         <v>103</v>
       </c>
@@ -4042,8 +4090,9 @@
       <c r="AT36" s="18"/>
       <c r="AU36" s="18"/>
       <c r="AV36" s="18"/>
+      <c r="AW36" s="18"/>
     </row>
-    <row r="37" spans="1:48" ht="31.2">
+    <row r="37" spans="1:49" ht="31.5">
       <c r="A37" s="21" t="s">
         <v>0</v>
       </c>
@@ -4106,8 +4155,9 @@
       <c r="AT37" s="18"/>
       <c r="AU37" s="18"/>
       <c r="AV37" s="18"/>
+      <c r="AW37" s="18"/>
     </row>
-    <row r="38" spans="1:48" ht="16.2" customHeight="1">
+    <row r="38" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A38" s="21" t="s">
         <v>0</v>
       </c>
@@ -4170,8 +4220,9 @@
       <c r="AT38" s="18"/>
       <c r="AU38" s="18"/>
       <c r="AV38" s="18"/>
+      <c r="AW38" s="18"/>
     </row>
-    <row r="39" spans="1:48" ht="16.2" customHeight="1">
+    <row r="39" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A39" s="21" t="s">
         <v>0</v>
       </c>
@@ -4232,8 +4283,9 @@
       <c r="AT39" s="18"/>
       <c r="AU39" s="18"/>
       <c r="AV39" s="18"/>
+      <c r="AW39" s="18"/>
     </row>
-    <row r="40" spans="1:48" ht="16.2" customHeight="1">
+    <row r="40" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A40" s="21" t="s">
         <v>0</v>
       </c>
@@ -4294,8 +4346,9 @@
       <c r="AT40" s="18"/>
       <c r="AU40" s="18"/>
       <c r="AV40" s="18"/>
+      <c r="AW40" s="18"/>
     </row>
-    <row r="41" spans="1:48" ht="16.2" customHeight="1">
+    <row r="41" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A41" s="21" t="s">
         <v>0</v>
       </c>
@@ -4356,8 +4409,9 @@
       <c r="AT41" s="18"/>
       <c r="AU41" s="18"/>
       <c r="AV41" s="18"/>
+      <c r="AW41" s="18"/>
     </row>
-    <row r="42" spans="1:48" ht="16.2" customHeight="1">
+    <row r="42" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A42" s="21" t="s">
         <v>0</v>
       </c>
@@ -4418,8 +4472,9 @@
       <c r="AT42" s="18"/>
       <c r="AU42" s="18"/>
       <c r="AV42" s="18"/>
+      <c r="AW42" s="18"/>
     </row>
-    <row r="43" spans="1:48" ht="16.2" customHeight="1">
+    <row r="43" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A43" s="24" t="s">
         <v>0</v>
       </c>
@@ -4480,8 +4535,9 @@
       <c r="AT43" s="19"/>
       <c r="AU43" s="19"/>
       <c r="AV43" s="19"/>
+      <c r="AW43" s="19"/>
     </row>
-    <row r="44" spans="1:48" ht="16.2" customHeight="1">
+    <row r="44" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
@@ -4490,7 +4546,7 @@
       <c r="J44" s="5"/>
       <c r="K44" s="5"/>
     </row>
-    <row r="45" spans="1:48" ht="22.95" customHeight="1">
+    <row r="45" spans="1:49" ht="22.9" customHeight="1">
       <c r="A45" s="6" t="s">
         <v>72</v>
       </c>
@@ -4555,8 +4611,9 @@
       <c r="AT45" s="7"/>
       <c r="AU45" s="7"/>
       <c r="AV45" s="7"/>
+      <c r="AW45" s="7"/>
     </row>
-    <row r="46" spans="1:48" ht="16.2" customHeight="1">
+    <row r="46" spans="1:49" ht="16.149999999999999" customHeight="1">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -4565,7 +4622,7 @@
       <c r="J46" s="5"/>
       <c r="K46" s="5"/>
     </row>
-    <row r="47" spans="1:48" ht="22.95" customHeight="1">
+    <row r="47" spans="1:49" ht="22.9" customHeight="1">
       <c r="A47" s="6" t="s">
         <v>72</v>
       </c>
@@ -4630,20 +4687,21 @@
       <c r="AT47" s="7"/>
       <c r="AU47" s="7"/>
       <c r="AV47" s="7"/>
+      <c r="AW47" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AV2" xr:uid="{344DF7D5-D639-4355-89FB-833EF1843A63}"/>
+  <autoFilter ref="A1:AW2" xr:uid="{344DF7D5-D639-4355-89FB-833EF1843A63}"/>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="F4:H47">
-    <cfRule type="expression" dxfId="3" priority="6">
-      <formula>LEN(D4)&gt;150</formula>
-    </cfRule>
+  <conditionalFormatting sqref="C1:C2">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3:C1048576">
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C2">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  <conditionalFormatting sqref="F4:H47">
+    <cfRule type="expression" dxfId="1" priority="6">
+      <formula>LEN(D4)&gt;150</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I4:I47">
     <cfRule type="expression" dxfId="0" priority="8">

</xml_diff>

<commit_message>
Correction bug - Merci à toute l'équipe de Gustave Eiffel pour le signalement !
</commit_message>
<xml_diff>
--- a/maquette-type.xlsx
+++ b/maquette-type.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apereir\Documents\En cours\En cours Maquettes\scripts\maquettes-xl2json\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apereir\Documents\En_cours\Scripts_Pegase\maquettes-xl2json\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E644C205-C610-4A76-A892-2B137B2B4E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B11A5D-BCA2-4925-9F2C-25F76FC17071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A6F31FBE-6D40-488E-B868-E7547D61F047}"/>
+    <workbookView xWindow="3555" yWindow="3210" windowWidth="17280" windowHeight="10005" xr2:uid="{A6F31FBE-6D40-488E-B868-E7547D61F047}"/>
   </bookViews>
   <sheets>
     <sheet name="Format complet" sheetId="1" r:id="rId1"/>
@@ -2339,6 +2339,7 @@
       <c r="AF9" s="18"/>
       <c r="AH9" s="18"/>
       <c r="AI9" s="32"/>
+      <c r="AJ9" s="18"/>
       <c r="AK9" s="18"/>
       <c r="AL9" s="18"/>
       <c r="AM9" s="18"/>

</xml_diff>